<commit_message>
#8 Parts selection in progress
</commit_message>
<xml_diff>
--- a/Design-Files/Receiver433MHz-v1.0/Deliverables/BOM/eSpark-BOM-Receiver_v1.0.xlsx
+++ b/Design-Files/Receiver433MHz-v1.0/Deliverables/BOM/eSpark-BOM-Receiver_v1.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\Receiver433MHz\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\hasanmehmood-motordriver\Design-Files\Receiver433MHz-v1.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="92">
   <si>
     <t>Component list</t>
   </si>
@@ -286,6 +286,15 @@
   </si>
   <si>
     <t>Receiver_v1.0.</t>
+  </si>
+  <si>
+    <t>AC0402BRNPO9BN2R4</t>
+  </si>
+  <si>
+    <t>CL05B104KO5VPNC</t>
+  </si>
+  <si>
+    <t>GCM1555C1H6R0DA16D</t>
   </si>
 </sst>
 </file>
@@ -749,7 +758,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -916,6 +925,9 @@
     <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -948,9 +960,7 @@
       <alignment horizontal="center" vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1293,7 +1303,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:S20"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
@@ -1314,9 +1324,10 @@
     <col min="17" max="17" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="22" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1327,17 +1338,17 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="62"/>
-      <c r="L1" s="62"/>
-      <c r="M1" s="62"/>
-      <c r="N1" s="62"/>
-      <c r="O1" s="62"/>
-      <c r="P1" s="62"/>
-      <c r="Q1" s="62"/>
-      <c r="R1" s="62"/>
-      <c r="S1" s="63"/>
+      <c r="K1" s="63"/>
+      <c r="L1" s="63"/>
+      <c r="M1" s="63"/>
+      <c r="N1" s="63"/>
+      <c r="O1" s="63"/>
+      <c r="P1" s="63"/>
+      <c r="Q1" s="63"/>
+      <c r="R1" s="63"/>
+      <c r="S1" s="64"/>
     </row>
-    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="21"/>
       <c r="C2" s="31"/>
@@ -1362,7 +1373,7 @@
       <c r="R2" s="4"/>
       <c r="S2" s="3"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="22"/>
       <c r="C3" s="32"/>
@@ -1385,9 +1396,9 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="64"/>
+      <c r="S3" s="65"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="22"/>
       <c r="C4" s="32"/>
@@ -1410,9 +1421,9 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="65"/>
+      <c r="S4" s="66"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="22"/>
       <c r="C5" s="32"/>
@@ -1435,9 +1446,9 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="65"/>
+      <c r="S5" s="66"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="23"/>
       <c r="C6" s="33"/>
@@ -1456,9 +1467,9 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="65"/>
+      <c r="S6" s="66"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="24"/>
       <c r="C7" s="34"/>
@@ -1477,9 +1488,9 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="65"/>
+      <c r="S7" s="66"/>
     </row>
-    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="27"/>
       <c r="C8" s="35"/>
@@ -1498,9 +1509,9 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="65"/>
+      <c r="S8" s="66"/>
     </row>
-    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:22" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="30" t="s">
         <v>4</v>
@@ -1557,7 +1568,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="36" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:22" ht="36" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
       <c r="B10" s="46">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -1612,8 +1623,14 @@
       </c>
       <c r="R10" s="37"/>
       <c r="S10" s="50"/>
+      <c r="U10" t="s">
+        <v>89</v>
+      </c>
+      <c r="V10" s="73" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
       <c r="B11" s="47">
         <f t="shared" ref="B11:B17" si="0">ROW(B11) - ROW($B$9)</f>
@@ -1668,8 +1685,14 @@
       </c>
       <c r="R11" s="51"/>
       <c r="S11" s="51"/>
+      <c r="U11" t="s">
+        <v>90</v>
+      </c>
+      <c r="V11" s="73" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="12" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:22" ht="24" x14ac:dyDescent="0.25">
       <c r="A12" s="1"/>
       <c r="B12" s="46">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -1724,8 +1747,14 @@
       </c>
       <c r="R12" s="37"/>
       <c r="S12" s="59"/>
+      <c r="U12" t="s">
+        <v>91</v>
+      </c>
+      <c r="V12" s="73" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="13" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:22" ht="48" x14ac:dyDescent="0.25">
       <c r="A13" s="1"/>
       <c r="B13" s="47">
         <f t="shared" si="0"/>
@@ -1743,7 +1772,7 @@
       <c r="F13" s="51" t="s">
         <v>34</v>
       </c>
-      <c r="G13" s="72" t="s">
+      <c r="G13" s="62" t="s">
         <v>81</v>
       </c>
       <c r="H13" s="51" t="s">
@@ -1780,8 +1809,11 @@
       </c>
       <c r="R13" s="51"/>
       <c r="S13" s="59"/>
+      <c r="V13" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="14" spans="1:19" ht="48" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:22" ht="48" x14ac:dyDescent="0.25">
       <c r="A14" s="1"/>
       <c r="B14" s="46">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -1799,7 +1831,7 @@
       <c r="F14" s="37" t="s">
         <v>35</v>
       </c>
-      <c r="G14" s="72" t="s">
+      <c r="G14" s="62" t="s">
         <v>86</v>
       </c>
       <c r="H14" s="51" t="s">
@@ -1836,8 +1868,11 @@
       </c>
       <c r="R14" s="37"/>
       <c r="S14" s="59"/>
+      <c r="V14" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="15" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:22" ht="24" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
       <c r="B15" s="47">
         <f t="shared" si="0"/>
@@ -1892,8 +1927,11 @@
       </c>
       <c r="R15" s="51"/>
       <c r="S15" s="59"/>
+      <c r="V15" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="16" spans="1:19" ht="24" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:22" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
       <c r="B16" s="46">
         <f>ROW(B16) - ROW($B$9)</f>
@@ -1948,8 +1986,11 @@
       </c>
       <c r="R16" s="37"/>
       <c r="S16" s="59"/>
+      <c r="V16" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
       <c r="B17" s="47">
         <f t="shared" si="0"/>
@@ -2004,8 +2045,11 @@
       </c>
       <c r="R17" s="51"/>
       <c r="S17" s="59"/>
+      <c r="V17" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="18" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:22" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="46">
         <f>ROW(B18) - ROW($B$9)</f>
@@ -2060,8 +2104,11 @@
       </c>
       <c r="R18" s="37"/>
       <c r="S18" s="39"/>
+      <c r="V18" t="s">
+        <v>80</v>
+      </c>
     </row>
-    <row r="19" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="40"/>
       <c r="C19" s="41"/>
@@ -2075,19 +2122,19 @@
       <c r="K19" s="45"/>
       <c r="L19" s="45"/>
       <c r="M19" s="45"/>
-      <c r="N19" s="70" t="s">
+      <c r="N19" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="O19" s="71"/>
-      <c r="P19" s="71"/>
+      <c r="O19" s="72"/>
+      <c r="P19" s="72"/>
       <c r="Q19" s="48">
         <f>SUM(Q10:Q18)</f>
         <v>4.5475999999999992</v>
       </c>
-      <c r="R19" s="66"/>
-      <c r="S19" s="67"/>
+      <c r="R19" s="67"/>
+      <c r="S19" s="68"/>
     </row>
-    <row r="20" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:22" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="25"/>
       <c r="C20" s="36"/>
@@ -2101,17 +2148,17 @@
       <c r="K20" s="10"/>
       <c r="L20" s="10"/>
       <c r="M20" s="10"/>
-      <c r="N20" s="70" t="s">
+      <c r="N20" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="O20" s="71"/>
-      <c r="P20" s="71"/>
+      <c r="O20" s="72"/>
+      <c r="P20" s="72"/>
       <c r="Q20" s="49">
         <f>Q19/5</f>
         <v>0.90951999999999988</v>
       </c>
-      <c r="R20" s="68"/>
-      <c r="S20" s="69"/>
+      <c r="R20" s="69"/>
+      <c r="S20" s="70"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2131,9 +2178,12 @@
     <hyperlink ref="O18" r:id="rId7"/>
     <hyperlink ref="O13" r:id="rId8"/>
     <hyperlink ref="O14" r:id="rId9"/>
+    <hyperlink ref="V10" r:id="rId10"/>
+    <hyperlink ref="V11" r:id="rId11"/>
+    <hyperlink ref="V12" r:id="rId12"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId10"/>
-  <drawing r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId13"/>
+  <drawing r:id="rId14"/>
 </worksheet>
 </file>
</xml_diff>